<commit_message>
Add the web app, prediction API, and Supabase storage.
</commit_message>
<xml_diff>
--- a/chem_excel_final.xlsx
+++ b/chem_excel_final.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jyothi\Chemistry\"/>
@@ -1735,9 +1735,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K102"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
+    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="10" width="6" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>

</xml_diff>